<commit_message>
Update AI Audit Log Slot4_Week2
</commit_message>
<xml_diff>
--- a/AI Audit Log_NghiemHoangPhuc.xlsx
+++ b/AI Audit Log_NghiemHoangPhuc.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fifa\CHUYÊN NGÀNH 7\SWD392\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fifa\CHUYÊN NGÀNH 7\SWD392\ai-audit-log-VuaCoder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88F00E6-A3CD-424B-90B1-4DF987C2460C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3A04F4-CEDE-4202-AE2B-81C45566E10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Week1" sheetId="2" r:id="rId2"/>
     <sheet name="Week2" sheetId="3" r:id="rId3"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId4"/>
+    <sheet name="Week3" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="47">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -254,6 +254,56 @@
   <si>
     <t>"Tức, nếu nó khởi tạo ra use case đó thì được tính là primary actor? Về phần tài liệu đó tôi hiểu rồi, nhưng có thêm phần này, hãy giải thích về quality attributes of SRS cho tôi, với mỗi phần cho 1 ví dụ thực tế sát dễ nắm hiểu và dễ hiểu được bản chất. LƯU Ý KHÔNG ĐƯỢC HALLUCATE để đảm bảo tính nhất quán (consistency), và sự khác biệt giữa extend và generalization như thế nào? Có từ khoá gì dễ phân biệt giữa 2 cái đó?"</t>
   </si>
+  <si>
+    <t>Slot4</t>
+  </si>
+  <si>
+    <t>"Tiếp tục, đến chương 7, hãy tổng kết cho tôi các kiến thức cụ thể, trọng tâm, với mỗi phần, phải đưa rõ phần lý thuyết nó nói về gì? ví dụ sát với thực tế nó sẽ như thế nào? và kết luận giúp rút ra được điều gì? tôi cần nắm rõ để có thể học hiểu 1 cách sâu nhất"</t>
+  </si>
+  <si>
+    <t>"Vậy association chỉ có chức năng cấu trúc 2 mối quan hệ xác định liên kết đối tượng này với đối tượng kia thôi? còn composition tức là nếu lớp A composition B thì cái nào bị phụ thuộc cái nào? Đồng thời aggregation thì A aggregation B thì cái nào phụ thuộc cái nào?"</t>
+  </si>
+  <si>
+    <t>"Tôi thấy hình như association của composition luôn là 1_1, còn phần aggegration luôn là 1_n, có phải vậy không? Hãy trả lời "ĐÚNG" hoặc "SAI", và giải thích vì sao 1 cách ngắn gọn"</t>
+  </si>
+  <si>
+    <t>"Ok đã hiểu. Đến phần quan hệ kế thừa và mô hình hoá, hãy giải thích các ý sau:
+- Generalization khác gì so với Specialization? Hay chỉ là cách gọi khác?
+- Và context modelling tôi chưa hiểu lắm, hãy giải thích kỹ hơn"</t>
+  </si>
+  <si>
+    <t>"À, tức là những phần mà mình có thể xác định được, những phần mình có thể tính toán được thì được tính là bên trong? còn bên ngoài là những thứ có thể thay đổi sao?"</t>
+  </si>
+  <si>
+    <t>"Ok, tức những thứ có sẵn ở thế giới và mình làm để giao tiếp với nó thì được tính là bên ngoài?
+còn những thứ mình phải làm để hệ thống hoạt động là bên trong?
+Vậy ví dụ:
+1 trang web của mình, và có chức năng login, thì người dùng là bên ngoài, và bên trong là thuật toán để trả về tài khoản người dùng đó hay sao?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI chia nhỏ các kiến thức cốt lõi của chương 7 theo đúng cấu trúc yêu cầu: Định nghĩa lý thuyết, lồng ghép ví dụ thực tế và rút ra bài học.
+Kiểm chứng: Cấu trúc trả lời logic và mạch lạc, tuân thủ đúng định dạng mà tôi yêu cầu. AI làm tốt việc đưa các kiến thức học thuật thành các case-study dễ hình dung, giúp việc học sâu hiệu quả hơn.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI xác nhận vai trò của Association, Composition và Aggegration
+Kiểm chứng: Lời giải thích ngắn gọn, đi thẳng vào việc đối tượng nào nắm quyền kiểm soát vòng đời của đối tượng nào.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI lập tức trả lời "SAI" như yêu cầu, đồng thời giải thích rằng những con số đó được quyết định bởi logic nghiệp vụ thực tế chứ không bị đóng khung cứng nhắc bởi loại quan hệ.
+Kiểm chứng: AI đưa kết luận chuẩn xác, đầy đủ, nắm rõ được các quy trình một cách trực quan, dễ hiểu do đã kèm với ví dụ. Sự khác biệt cũng được chỉ rõ khi AI đưa ra những từ khoá giúp tôi có thể hiểu và nắm rõ.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích và điều chỉnh lại cách hiểu này, giải thích không dựa vào tính cố định hay biến đổi, mà dựa vào việc phần mềm của mình có quyền kiểm soát và xử lý nó hay không.
+Kiểm chứng: AI thể hiện sự nhạy bén khi nhận ra người dùng đang suy luận chệch hướng.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phân tích Generalization và Specialization. Kế tiếp, AI làm rõ Context modelling là việc vạch ra ranh giới hệ thống.
+Kiểm chứng: Cách so sánh hai thuật ngữ rất trực quan, giúp tôi không bị rối rắm bởi từ ngữ.</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI thể hiện sự đồng tình cao độ và dùng chính ví dụ Login để bóc tách.
+Kiểm chứng: Lời khen ngợi kịp thời giúp củng cố sự tự tin của người học. Việc phân tích mổ xẻ ví dụ thực tế đã chốt lại một cách thuyết phục toàn bộ khái niệm trừu tượng về Context Diagram.</t>
+  </si>
 </sst>
 </file>
 
@@ -332,7 +382,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -368,21 +418,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -910,7 +945,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A16565-6ACB-4DDB-B0C1-55C7722368A3}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="4.625" bestFit="1" customWidth="1"/>
@@ -937,7 +972,7 @@
       <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="13" t="s">
         <v>27</v>
       </c>
       <c r="C2" s="10" t="s">
@@ -975,19 +1010,92 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="13"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="16"/>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="13"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="17"/>
+    <row r="5" spans="1:4" ht="142.5">
+      <c r="A5" s="8">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="142.5">
+      <c r="A6" s="8">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="114">
+      <c r="A7" s="8">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="128.25">
+      <c r="A8" s="8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="85.5">
+      <c r="A9" s="8">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="199.5">
+      <c r="A10" s="8">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update Readme.md - Week3
</commit_message>
<xml_diff>
--- a/AI Audit Log_NghiemHoangPhuc.xlsx
+++ b/AI Audit Log_NghiemHoangPhuc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fifa\CHUYÊN NGÀNH 7\SWD392\ai-audit-log-VuaCoder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84C4140D-58F4-4022-A971-96835EEF6BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E807532F-F70B-4791-A40B-E256044F0E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="69">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -341,6 +341,44 @@
   <si>
     <t>Phản hồi: Code viết để làm cầu nối thì dùng nhãn &lt;&lt;user interaction&gt;&gt; hoặc &lt;&lt;proxy&gt;&gt;. Còn những gì thuộc thế giới vật lý bên ngoài (người thật, phần cứng) thì mới thêm chữ &lt;&lt;external&gt;&gt;.
 Kiểm chứng: Nắm được quy tắc này giúp tôi gỡ rối hoàn toàn khi vẽ biểu đồ.</t>
+  </si>
+  <si>
+    <t>Slot6</t>
+  </si>
+  <si>
+    <t>"Hãy giảng cho tôi về slide ch09-11 đó cho tôi, kèm theo các ví dụ trực quan, dễ hiểu, dễ liên tưởng và thực tế, ngoài đời, yêu cầu không được nói lang mang, nói quá dài dòng, nói đúng trọng điểm, những điều cần nhớ, và không được hallucate. Hãy ghi nhớ"</t>
+  </si>
+  <si>
+    <t>Phản hồi:Tổng quan về mô hình tương tác động (Dynamic Interaction) giữa các đối tượng trong hệ thống.
+Kiểm chứng: Bắt đầu chuyển từ tư duy "hệ thống có những gì" sang "chúng tương tác với nhau thế nào".</t>
+  </si>
+  <si>
+    <t>Phản hồi: Phân biệt 2 loại hành vi: Stateless (không phụ thuộc trạng thái) và State-dependent (phụ thuộc trạng thái).
+Kiểm chứng: Nắm được định nghĩa cơ bản. Cần phải phân biệt rạch ròi hai khái niệm này để lên luồng nghiệp vụ không bị sai logic.</t>
+  </si>
+  <si>
+    <t>"Giải thích rõ hơn ở phần stateless và state-dependent đi, đồng thời cho ví dụ cho thấy sự khác biệt của 2 cái đó"</t>
+  </si>
+  <si>
+    <t>"À, tức stateless sẽ không ghi nhớ bộ nhớ hôm qua đã làm gì, làm như thế nào, còn state-dependent sẽ ghi nhớ lịch sử đó hả?"</t>
+  </si>
+  <si>
+    <t>"Vậy làm sao để phân biệt những hành động mang tính stateless, mang tính state-dependent"</t>
+  </si>
+  <si>
+    <t>"Tôi hiểu rồi, vậy còn cách vẽ? Nãy bạn chưa giải thích cho tôi"</t>
+  </si>
+  <si>
+    <t>Phản hồi: Xác nhận đúng. Stateless làm xong là quên (không lưu trạng thái). State-dependent ghi nhớ lịch sử để quyết định hành động tiếp theo.
+Kiểm chứng: Giúp liên tưởng và phân biệt rõ của stateless và state-dependent</t>
+  </si>
+  <si>
+    <t>Phản hồi: Nếu quyết định bước tiếp theo đòi hỏi phải kiểm tra "quá khứ/trạng thái hiện tại", đó là State-dependent. Ngược lại là Stateless.
+Kiểm chứng: Đây chính là công thức vàng khi làm Use Case. Cứ đọc tài liệu specification, nếu thấy có điều kiện kiểu "Chỉ cho phép thanh toán nếu đơn đang ở trạng thái X", thì tự động biết phải thiết kế theo cụm State-dependent.</t>
+  </si>
+  <si>
+    <t>Phản hồi: Hướng dẫn các bước vẽ sơ đồ. Nhấn mạnh 2 quy tắc: Phải khớp 100% tên event với biểu đồ Statechart, và nên vẽ tách luồng (Instance form) thay vì gộp chung (Generic form).
+Kiểm chứng: inh nghiệm xương máu cho việc làm tài liệu! Thay vì nhồi nhét đủ thứ If/Else (luồng đúng + luồng lỗi) vào chung một biểu đồ gây rối mắt, từ nay tôi sẽ tách rạch ròi luồng happy-path riêng và các luồng báo lỗi riêng</t>
   </si>
 </sst>
 </file>
@@ -1140,7 +1178,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="4.625" bestFit="1" customWidth="1"/>
@@ -1233,7 +1271,79 @@
         <v>57</v>
       </c>
     </row>
+    <row r="7" spans="1:4" ht="142.5">
+      <c r="A7" s="13">
+        <v>6</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="71.25">
+      <c r="A8" s="13">
+        <v>7</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="71.25">
+      <c r="A9" s="13">
+        <v>8</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="99.75">
+      <c r="A10" s="13">
+        <v>9</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="114">
+      <c r="A11" s="13">
+        <v>10</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>